<commit_message>
Update industrial sector (factoriescap_s) 0.xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/industrial sector (factoriescap_s) 0.xlsx
+++ b/clustering/sepsectors/industrial sector (factoriescap_s) 0.xlsx
@@ -211,6 +211,8 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2439,6 +2441,54 @@
     <sortCondition descending="1" ref="D2:D73"/>
   </sortState>
   <conditionalFormatting sqref="D77:D78">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E77:E78">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F77:F78">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G77:G78">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D73">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -2450,7 +2500,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E77:E78">
+  <conditionalFormatting sqref="E2:E73">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -2462,7 +2512,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F77:F78">
+  <conditionalFormatting sqref="F2:F73">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -2474,7 +2524,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G77:G78">
+  <conditionalFormatting sqref="G2:G73">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>